<commit_message>
feat: improve grammar templates and placeholder data for example generation
- Refined sentence structures in rule engine templates for better linguistic accuracy
- Enhanced fake data generation in placeholders to produce more realistic examples
- Supports improved clarity and diversity in Text2SQL output samples
</commit_message>
<xml_diff>
--- a/Text2SQL_Template/output/ddq_autogen_customer_account.xlsx
+++ b/Text2SQL_Template/output/ddq_autogen_customer_account.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="77">
   <si>
     <t>document</t>
   </si>
@@ -31,360 +31,284 @@
     <t>metadata</t>
   </si>
   <si>
-    <t>Tra cứu customer_account theo id</t>
-  </si>
-  <si>
-    <t>Tra cứu customer_account theo core_customer_id</t>
-  </si>
-  <si>
-    <t>Tra cứu customer_account theo account_no</t>
-  </si>
-  <si>
-    <t>Lọc customer_account theo account_class</t>
-  </si>
-  <si>
-    <t>Tra cứu customer_account theo order_no</t>
-  </si>
-  <si>
-    <t>Lọc customer_account theo status</t>
-  </si>
-  <si>
-    <t>Lọc customer_account theo verify_status</t>
-  </si>
-  <si>
-    <t>Lọc customer_account theo check_status</t>
-  </si>
-  <si>
-    <t>Tra cứu customer_account theo channel_id</t>
-  </si>
-  <si>
-    <t>Tra cứu customer_account theo khoảng thời gian (create_date)</t>
-  </si>
-  <si>
-    <t>Tra cứu customer_account theo account_branch</t>
-  </si>
-  <si>
-    <t>Tra cứu customer_account theo card_mask</t>
-  </si>
-  <si>
-    <t>Tra cứu customer_account theo customer_no</t>
-  </si>
-  <si>
-    <t>Tra cứu customer_account theo system_id</t>
-  </si>
-  <si>
-    <t>Tra cứu customer_account theo khoảng thời gian (end_date)</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác bản ghi dựa trên id</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác bản ghi dựa trên core_customer_id</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác bản ghi dựa trên account_no</t>
-  </si>
-  <si>
-    <t>Liệt kê danh sách theo tiêu chí account_class</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác bản ghi dựa trên order_no</t>
-  </si>
-  <si>
-    <t>Liệt kê danh sách theo tiêu chí status</t>
-  </si>
-  <si>
-    <t>Liệt kê danh sách theo tiêu chí verify_status</t>
-  </si>
-  <si>
-    <t>Liệt kê danh sách theo tiêu chí check_status</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác bản ghi dựa trên channel_id</t>
-  </si>
-  <si>
-    <t>Lọc dữ liệu phát sinh trong một khoảng ngày giờ</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác bản ghi dựa trên account_branch</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác bản ghi dựa trên card_mask</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác bản ghi dựa trên customer_no</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác bản ghi dựa trên system_id</t>
-  </si>
-  <si>
-    <t>Xem chi tiết biến động số dư tại số {{{id}}}
-Cho tôi xem lệnh chuyển tiền mang khóa chính {{{id}}}
-Tra cứu giao dịch tại mã {{{id}}}
-Kiểm tra biến động số dư có mã {{{id}}}
-Search biến động số dư theo primary key {{{id}}}
-Tra cứu giao dịch của số {{{id}}}
-Cho tôi xem giao dịch với id {{{id}}}
-Tra cứu biến động số dư theo số {{{id}}}
-Hiển thị giao dịch mang id {{{id}}}
-Tra cứu giao dịch tại số {{{id}}}
-Hiển thị lệnh chuyển tiền với khóa chính {{{id}}}
-Tìm biến động số dư với số {{{id}}}
-Tra cứu history tại khóa chính {{{id}}}
-Liệt kê lệnh chuyển tiền của mã {{{id}}}
-mã {{{id}}} là bao nhiêu</t>
-  </si>
-  <si>
-    <t>Xem chi tiết biến động số dư tại số {{{core_customer_id}}}
-Tra cứu giao dịch tại mã {{{core_customer_id}}}
-Cho tôi xem biến động số dư có id khách hàng bên lõi {{{core_customer_id}}}
-Kiểm tra biến động số dư có mã {{{core_customer_id}}}
-Tìm lệnh chuyển tiền tại id khách hàng bên lõi {{{core_customer_id}}}
-Kiểm tra history của id khách hàng bên lõi {{{core_customer_id}}}
-Tra cứu giao dịch của số {{{core_customer_id}}}
-Cho tôi xem giao dịch với id {{{core_customer_id}}}
-Search giao dịch mang id khách hàng bên lõi {{{core_customer_id}}}
-Tra cứu biến động số dư theo số {{{core_customer_id}}}
-Hiển thị giao dịch mang id {{{core_customer_id}}}
-Tra cứu giao dịch tại số {{{core_customer_id}}}
-Cho tôi xem history có core banking {{{core_customer_id}}}
-Tìm biến động số dư với số {{{core_customer_id}}}
-Kiểm tra history tại id khách hàng bên lõi {{{core_customer_id}}}</t>
-  </si>
-  <si>
-    <t>Search biến động số dư của số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch. {{{account_no}}}
-Cho tôi xem lệnh chuyển tiền tại số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch. {{{account_no}}}
-Xem chi tiết history của số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch. {{{account_no}}}
-Kiểm tra lệnh chuyển tiền mang số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch. {{{account_no}}}
-Xem chi tiết lệnh chuyển tiền của số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch. {{{account_no}}}
-Kiểm tra lệnh chuyển tiền của số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch. {{{account_no}}}
-Search lệnh chuyển tiền với số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch. {{{account_no}}}
-Tìm giao dịch tại số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch. {{{account_no}}}
-Tra cứu biến động số dư mang số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch. {{{account_no}}}
-Tìm biến động số dư tại số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch. {{{account_no}}}
-Liệt kê lệnh chuyển tiền với số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch. {{{account_no}}}
-Tìm history mang số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch. {{{account_no}}}
-số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch. {{{account_no}}} là bao nhiêu
-Tìm lệnh chuyển tiền theo số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch. {{{account_no}}}
-Tìm giao dịch của số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch. {{{account_no}}}</t>
-  </si>
-  <si>
-    <t>Lọc các history với ví dụ: tài khoản thanh toán, tài khoản tiết kiệm, thẻ tín dụng... {{{account_class}}}
-Lọc các biến động số dư của phân loại tài khoản {{{account_class}}}
-Danh sách giao dịch của phân loại tài khoản {{{account_class}}}
-Danh sách lệnh chuyển tiền có ví dụ: tài khoản thanh toán, tài khoản tiết kiệm, thẻ tín dụng... {{{account_class}}}
-Danh sách lệnh chuyển tiền mang phân loại tài khoản {{{account_class}}}
-Danh sách biến động số dư theo phân loại tài khoản {{{account_class}}}
-Những biến động số dư có ví dụ: tài khoản thanh toán, tài khoản tiết kiệm, thẻ tín dụng... {{{account_class}}}
-Các history có ví dụ: tài khoản thanh toán, tài khoản tiết kiệm, thẻ tín dụng... {{{account_class}}}
-Lọc các giao dịch của ví dụ: tài khoản thanh toán, tài khoản tiết kiệm, thẻ tín dụng... {{{account_class}}}
-Các giao dịch với ví dụ: tài khoản thanh toán, tài khoản tiết kiệm, thẻ tín dụng... {{{account_class}}}
-Danh sách lệnh chuyển tiền của ví dụ: tài khoản thanh toán, tài khoản tiết kiệm, thẻ tín dụng... {{{account_class}}}
-Các lệnh chuyển tiền có ví dụ: tài khoản thanh toán, tài khoản tiết kiệm, thẻ tín dụng... {{{account_class}}}
-Lọc các lệnh chuyển tiền của ví dụ: tài khoản thanh toán, tài khoản tiết kiệm, thẻ tín dụng... {{{account_class}}}
-Những biến động số dư mang phân loại tài khoản {{{account_class}}}
-Các history theo ví dụ: tài khoản thanh toán, tài khoản tiết kiệm, thẻ tín dụng... {{{account_class}}}</t>
-  </si>
-  <si>
-    <t>Tra cứu lệnh chuyển tiền mang app/web {{{order_no}}}
-Liệt kê biến động số dư có số thứ tự hiển thị tài khoản trên giao diện {{{order_no}}}
-Tra cứu history mang app/web {{{order_no}}}
-Search giao dịch có số thứ tự hiển thị tài khoản trên giao diện {{{order_no}}}
-Kiểm tra giao dịch với số thứ tự hiển thị tài khoản trên giao diện {{{order_no}}}
-Tìm giao dịch theo số thứ tự hiển thị tài khoản trên giao diện {{{order_no}}}
-Tìm giao dịch mang app/web {{{order_no}}}
-Search giao dịch tại app/web {{{order_no}}}
-Tìm lệnh chuyển tiền của số thứ tự hiển thị tài khoản trên giao diện {{{order_no}}}
-Kiểm tra biến động số dư với số thứ tự hiển thị tài khoản trên giao diện {{{order_no}}}
-Hiển thị history mang số thứ tự hiển thị tài khoản trên giao diện {{{order_no}}}
-Liệt kê giao dịch tại số thứ tự hiển thị tài khoản trên giao diện {{{order_no}}}
-Kiểm tra history theo app/web {{{order_no}}}
-Tra cứu biến động số dư có app/web {{{order_no}}}
-Liệt kê history theo app/web {{{order_no}}}</t>
-  </si>
-  <si>
-    <t>Những lệnh chuyển tiền mang kết quả {{{status}}}
-Lọc các biến động số dư của trạng thái {{{status}}}
-Danh sách history với ví dụ: a - active, i - inactive, c - closed {{{status}}}
-Danh sách history theo trạng thái tài khoản {{{status}}}
-Lọc các biến động số dư có ví dụ: a - active, i - inactive, c - closed {{{status}}}
-Lọc các lệnh chuyển tiền mang kết quả {{{status}}}
-Các lệnh chuyển tiền tại trạng thái tài khoản {{{status}}}
-Lọc các history có trạng thái tài khoản {{{status}}}
-Các giao dịch mang trạng thái tài khoản {{{status}}}
-Những biến động số dư theo tình trạng {{{status}}}
-Các giao dịch theo ví dụ: a - active, i - inactive, c - closed {{{status}}}
-Các giao dịch mang ví dụ: a - active, i - inactive, c - closed {{{status}}}
-Danh sách biến động số dư của trạng thái {{{status}}}
-Những giao dịch của kết quả {{{status}}}
-Lọc các lệnh chuyển tiền của ví dụ: a - active, i - inactive, c - closed {{{status}}}</t>
-  </si>
-  <si>
-    <t>Lọc các history có trạng thái xác thực tài khoản {{{verify_status}}}
-Những lệnh chuyển tiền mang kết quả {{{verify_status}}}
-Lọc các biến động số dư của trạng thái {{{verify_status}}}
-Những history của đã xác minh thông tin hay chưa {{{verify_status}}}
-Lọc các lệnh chuyển tiền mang kết quả {{{verify_status}}}
-Những history mang đã xác minh thông tin hay chưa {{{verify_status}}}
-Lọc các lệnh chuyển tiền có trạng thái xác thực tài khoản {{{verify_status}}}
-Những biến động số dư theo tình trạng {{{verify_status}}}
-Các history với đã xác minh thông tin hay chưa {{{verify_status}}}
-Danh sách biến động số dư của trạng thái {{{verify_status}}}
-Những giao dịch của kết quả {{{verify_status}}}
-Lọc các biến động số dư theo trạng thái xác thực tài khoản {{{verify_status}}}
-Danh sách giao dịch theo kết quả {{{verify_status}}}
-Các lệnh chuyển tiền của tình trạng {{{verify_status}}}
-Các giao dịch mang tình trạng {{{verify_status}}}</t>
-  </si>
-  <si>
-    <t>Những lệnh chuyển tiền tại trạng thái kiểm tra {{{check_status}}}
-Lọc các biến động số dư của trạng thái {{{check_status}}}
-Những lệnh chuyển tiền mang kết quả {{{check_status}}}
-Các history tại trạng thái kiểm tra {{{check_status}}}
-Lọc các giao dịch theo mặc định 'u' - unknown hoặc unchecked {{{check_status}}}
-Lọc các lệnh chuyển tiền mang kết quả {{{check_status}}}
-Lọc các history có mặc định 'u' - unknown hoặc unchecked {{{check_status}}}
-Những giao dịch có trạng thái kiểm tra {{{check_status}}}
-Danh sách history mang mặc định 'u' - unknown hoặc unchecked {{{check_status}}}
-Những biến động số dư theo tình trạng {{{check_status}}}
-Các lệnh chuyển tiền của trạng thái kiểm tra {{{check_status}}}
-Danh sách biến động số dư của trạng thái {{{check_status}}}
-Những giao dịch của kết quả {{{check_status}}}
-Danh sách giao dịch theo kết quả {{{check_status}}}
-Danh sách lệnh chuyển tiền theo trạng thái kiểm tra {{{check_status}}}</t>
-  </si>
-  <si>
-    <t>Xem chi tiết biến động số dư tại số {{{channel_id}}}
-Tra cứu giao dịch của số {{{channel_id}}}
-Hiển thị giao dịch mang id {{{channel_id}}}
-Tìm biến động số dư với số {{{channel_id}}}
-Liệt kê giao dịch mang ví dụ: mobile, internet banking, quầy giao dịch {{{channel_id}}}
-Tra cứu lệnh chuyển tiền mang nguồn {{{channel_id}}}
-Search biến động số dư theo mã {{{channel_id}}}
-Kiểm tra giao dịch tại ví dụ: mobile, internet banking, quầy giao dịch {{{channel_id}}}
-Tìm lệnh chuyển tiền của id kênh tạo tài khoản {{{channel_id}}}
-Cho tôi xem giao dịch của kênh {{{channel_id}}}
-Liệt kê lệnh chuyển tiền tại số {{{channel_id}}}
-Cho tôi xem biến động số dư mang ví dụ: mobile, internet banking, quầy giao dịch {{{channel_id}}}
-Tìm history tại id {{{channel_id}}}
-Xem chi tiết history với mã {{{channel_id}}}
-Cho tôi xem biến động số dư với kênh {{{channel_id}}}</t>
-  </si>
-  <si>
-    <t>Sao kê giao dịch từ ngày {{start_date}} đến {{end_date}}
-Liệt kê lịch sử trong khoảng thời gian {{start_date}} - {{end_date}}
-Kiểm tra giao dịch phát sinh từ {{start_date}} tới {{end_date}}
-Cho tôi xem biến động số dư giữa {{start_date}} và {{end_date}}</t>
-  </si>
-  <si>
-    <t>Hiển thị lệnh chuyển tiền tại mã chi nhánh nơi quản lý tài khoản này. {{{account_branch}}}
-Cho tôi xem history có mã chi nhánh nơi quản lý tài khoản này. {{{account_branch}}}
-Hiển thị lệnh chuyển tiền mang mã chi nhánh nơi quản lý tài khoản này. {{{account_branch}}}
-Liệt kê giao dịch tại mã chi nhánh nơi quản lý tài khoản này. {{{account_branch}}}
-Hiển thị lệnh chuyển tiền theo mã chi nhánh nơi quản lý tài khoản này. {{{account_branch}}}
-Hiển thị history theo mã chi nhánh nơi quản lý tài khoản này. {{{account_branch}}}
-Hiển thị history tại mã chi nhánh nơi quản lý tài khoản này. {{{account_branch}}}
-Cho tôi xem history mang mã chi nhánh nơi quản lý tài khoản này. {{{account_branch}}}
-Tìm history theo mã chi nhánh nơi quản lý tài khoản này. {{{account_branch}}}
-Xem chi tiết biến động số dư mang mã chi nhánh nơi quản lý tài khoản này. {{{account_branch}}}
-Search biến động số dư có mã chi nhánh nơi quản lý tài khoản này. {{{account_branch}}}
-Kiểm tra history mang mã chi nhánh nơi quản lý tài khoản này. {{{account_branch}}}
-Liệt kê giao dịch có mã chi nhánh nơi quản lý tài khoản này. {{{account_branch}}}
-Tìm biến động số dư mang mã chi nhánh nơi quản lý tài khoản này. {{{account_branch}}}
-Liệt kê giao dịch của mã chi nhánh nơi quản lý tài khoản này. {{{account_branch}}}</t>
-  </si>
-  <si>
-    <t>Hiển thị giao dịch mang ví dụ: 411122****1234 {{{card_mask}}}
-Liệt kê lệnh chuyển tiền theo ví dụ: 411122****1234 {{{card_mask}}}
-Hiển thị history có số thẻ được che bớt {{{card_mask}}}
-Liệt kê history tại số thẻ được che bớt {{{card_mask}}}
-Kiểm tra giao dịch theo số thẻ được che bớt {{{card_mask}}}
-Search giao dịch có ví dụ: 411122****1234 {{{card_mask}}}
-Tra cứu biến động số dư có ví dụ: 411122****1234 {{{card_mask}}}
-Hiển thị biến động số dư mang số thẻ được che bớt {{{card_mask}}}
-Search biến động số dư có số thẻ được che bớt {{{card_mask}}}
-Cho tôi xem biến động số dư với ví dụ: 411122****1234 {{{card_mask}}}
-Cho tôi xem biến động số dư mang số thẻ được che bớt {{{card_mask}}}
-Liệt kê giao dịch tại ví dụ: 411122****1234 {{{card_mask}}}
-Hiển thị lệnh chuyển tiền mang số thẻ được che bớt {{{card_mask}}}
-Liệt kê biến động số dư với số thẻ được che bớt {{{card_mask}}}
-Xem chi tiết biến động số dư có số thẻ được che bớt {{{card_mask}}}</t>
-  </si>
-  <si>
-    <t>Hiển thị history theo mã số khách hàng {{{customer_no}}}
-Xem chi tiết biến động số dư có customer number {{{customer_no}}}
-Kiểm tra biến động số dư theo customer number {{{customer_no}}}
-Tra cứu history với customer number {{{customer_no}}}
-Tìm biến động số dư của mã số khách hàng {{{customer_no}}}
-Xem chi tiết biến động số dư có mã số khách hàng {{{customer_no}}}
-Xem chi tiết lệnh chuyển tiền tại mã số khách hàng {{{customer_no}}}
-Tra cứu lệnh chuyển tiền của customer number {{{customer_no}}}
-Tìm history với mã số khách hàng {{{customer_no}}}
-Tìm lệnh chuyển tiền theo mã số khách hàng {{{customer_no}}}
-Kiểm tra lệnh chuyển tiền mang customer number {{{customer_no}}}
-Hiển thị biến động số dư với customer number {{{customer_no}}}
-Tìm history với customer number {{{customer_no}}}
-Kiểm tra history với mã số khách hàng {{{customer_no}}}
-Tìm biến động số dư theo customer number {{{customer_no}}}</t>
-  </si>
-  <si>
-    <t>Xem chi tiết biến động số dư tại số {{{system_id}}}
-Tra cứu giao dịch tại mã {{{system_id}}}
-Kiểm tra biến động số dư có mã {{{system_id}}}
-Tra cứu giao dịch của số {{{system_id}}}
-Cho tôi xem giao dịch với id {{{system_id}}}
-Tra cứu biến động số dư theo số {{{system_id}}}
-Hiển thị giao dịch mang id {{{system_id}}}
-Tra cứu giao dịch tại số {{{system_id}}}
-Tìm biến động số dư với số {{{system_id}}}
-Liệt kê lệnh chuyển tiền của mã {{{system_id}}}
-mã {{{system_id}}} là bao nhiêu
-Liệt kê giao dịch mang mã nguồn cung cấp dữ liệu tài khoản này. {{{system_id}}}
-Tra cứu lệnh chuyển tiền tại mã {{{system_id}}}
-Tra cứu giao dịch có mã {{{system_id}}}
-Search biến động số dư theo mã {{{system_id}}}</t>
-  </si>
-  <si>
-    <t>id, tra cứu, tìm kiếm</t>
-  </si>
-  <si>
-    <t>core_customer_id, tra cứu, tìm kiếm</t>
-  </si>
-  <si>
-    <t>account_no, tra cứu, tìm kiếm</t>
-  </si>
-  <si>
-    <t>account_class, danh sách, lọc</t>
-  </si>
-  <si>
-    <t>order_no, tra cứu, tìm kiếm</t>
-  </si>
-  <si>
-    <t>status, danh sách, lọc</t>
-  </si>
-  <si>
-    <t>verify_status, danh sách, lọc</t>
-  </si>
-  <si>
-    <t>check_status, danh sách, lọc</t>
-  </si>
-  <si>
-    <t>channel_id, tra cứu, tìm kiếm</t>
-  </si>
-  <si>
-    <t>thời gian, ngày tháng, sao kê</t>
-  </si>
-  <si>
-    <t>account_branch, tra cứu, tìm kiếm</t>
-  </si>
-  <si>
-    <t>card_mask, tra cứu, tìm kiếm</t>
-  </si>
-  <si>
-    <t>customer_no, tra cứu, tìm kiếm</t>
-  </si>
-  <si>
-    <t>system_id, tra cứu, tìm kiếm</t>
+    <t>customer_account | Tra cứu theo khóa chính</t>
+  </si>
+  <si>
+    <t>customer_account | Tra cứu theo số</t>
+  </si>
+  <si>
+    <t>customer_account | Tra cứu theo số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch.</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc theo ví dụ: tài khoản thanh toán, tài khoản tiết kiệm, thẻ tín dụng...</t>
+  </si>
+  <si>
+    <t>customer_account | Tra cứu theo số thứ tự hiển thị tài khoản trên giao diện</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc theo trạng thái tài khoản</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc theo kết quả</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc theo trạng thái kiểm tra</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc theo thời gian (hôm)</t>
+  </si>
+  <si>
+    <t>customer_account | Tra cứu theo mã chi nhánh nơi quản lý tài khoản này.</t>
+  </si>
+  <si>
+    <t>customer_account | Tra cứu theo ví dụ: 411122****1234</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc account_class theo Thời gian</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác tài khoản dựa trên khóa chính</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác tài khoản dựa trên số</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác tài khoản dựa trên số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch.</t>
+  </si>
+  <si>
+    <t>Liệt kê danh sách tài khoản theo nhóm ví dụ: tài khoản thanh toán, tài khoản tiết kiệm, thẻ tín dụng...</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác tài khoản dựa trên số thứ tự hiển thị tài khoản trên giao diện</t>
+  </si>
+  <si>
+    <t>Liệt kê danh sách tài khoản theo nhóm trạng thái tài khoản</t>
+  </si>
+  <si>
+    <t>Liệt kê danh sách tài khoản theo nhóm kết quả</t>
+  </si>
+  <si>
+    <t>Liệt kê danh sách tài khoản theo nhóm trạng thái kiểm tra</t>
+  </si>
+  <si>
+    <t>Sao kê lịch sử tài khoản trong khoảng thời gian</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác tài khoản dựa trên mã chi nhánh nơi quản lý tài khoản này.</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác tài khoản dựa trên ví dụ: 411122****1234</t>
+  </si>
+  <si>
+    <t>Kết hợp lọc theo account_class và khoảng ngày tháng</t>
+  </si>
+  <si>
+    <t>Vui lòng Tra cứu thông tin chi tiết của tài khoản có khóa chính là 87973
+Tra cứu tài khoản theo khóa chính 31884
+Thông tin về tài khoản số 64994
+tài khoản 59395
+Xem chi tiết 2699
+Check khóa chính 17023
+khóa chính 19556 là của ai?
+Tìm kiếm tài khoản ứng với số 40512
+Hãy hiển thị dữ liệu bản ghi tài khoản với khóa chính 39125</t>
+  </si>
+  <si>
+    <t>Thông tin về tài khoản số 62473
+số 95126 là của ai?
+Vui lòng Tra cứu thông tin chi tiết của tài khoản có số là 6092
+Xem chi tiết 81370
+Hãy hiển thị dữ liệu bản ghi tài khoản với số 64097
+tài khoản 4826
+Check số 6141
+Tra cứu tài khoản theo số 8344
+Tìm kiếm tài khoản ứng với số 52165</t>
+  </si>
+  <si>
+    <t>Thông tin về tài khoản số 2654145137383
+Tìm kiếm tài khoản ứng với số 8126379878689
+Vui lòng Tra cứu thông tin chi tiết của tài khoản có số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch. là 9714958754928
+tài khoản 3484804855204
+số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch. 1309894317932 là của ai?
+Xem chi tiết 3098638162410
+Tra cứu tài khoản theo số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch. 9588891936675
+Hãy hiển thị dữ liệu bản ghi tài khoản với số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch. 5760431701535
+Check số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch. 930788480979</t>
+  </si>
+  <si>
+    <t>Hãy liệt kê danh sách các tài khoản có ví dụ: tài khoản thanh toán, tài khoản tiết kiệm, thẻ tín dụng... là khi
+Tìm tất cả tài khoản loại đi
+Danh sách nhưng
+Trích xuất báo cáo các tài khoản thuộc loại của
+Những tài khoản nào là của?
+Lọc các tài khoản đang ở trạng thái như
+Cho xem danh sách tài khoản với</t>
+  </si>
+  <si>
+    <t>Vui lòng Tra cứu thông tin chi tiết của tài khoản có số thứ tự hiển thị tài khoản trên giao diện là 79343
+số thứ tự hiển thị tài khoản trên giao diện 59019 là của ai?
+Xem chi tiết 14104
+Hãy hiển thị dữ liệu bản ghi tài khoản với số thứ tự hiển thị tài khoản trên giao diện 63043
+Tra cứu tài khoản theo số thứ tự hiển thị tài khoản trên giao diện 23900
+Thông tin về tài khoản số 62262
+tài khoản 69251
+Tìm kiếm tài khoản ứng với số 52271
+Check số thứ tự hiển thị tài khoản trên giao diện 61451</t>
+  </si>
+  <si>
+    <t>Lọc các tài khoản đang ở trạng thái dưới
+Hãy liệt kê danh sách các tài khoản có trạng thái tài khoản là điều
+Trích xuất báo cáo các tài khoản thuộc loại không
+Cho xem danh sách tài khoản chưa
+Những tài khoản nào là các?
+Tìm tất cả tài khoản loại giống
+Danh sách tại</t>
+  </si>
+  <si>
+    <t>Danh sách từng
+Lọc các tài khoản đang ở trạng thái với
+Cho xem danh sách tài khoản chỉ
+Hãy liệt kê danh sách các tài khoản có kết quả là chưa
+Tìm tất cả tài khoản loại gần
+Những tài khoản nào là với?
+Trích xuất báo cáo các tài khoản thuộc loại như</t>
+  </si>
+  <si>
+    <t>Hãy liệt kê danh sách các tài khoản có trạng thái kiểm tra là sẽ
+Lọc các tài khoản đang ở trạng thái từ
+Tìm tất cả tài khoản loại nhiều
+Cho xem danh sách tài khoản các
+Trích xuất báo cáo các tài khoản thuộc loại thay
+Những tài khoản nào là là?
+Danh sách thế</t>
+  </si>
+  <si>
+    <t>Tìm kiếm tài khoản ứng với số 43945
+Hãy hiển thị dữ liệu bản ghi tài khoản với số 36719
+số 74294 là của ai?
+Check số 66848
+Thông tin về tài khoản số 4811
+tài khoản 92320
+Tra cứu tài khoản theo số 64792
+Vui lòng Tra cứu thông tin chi tiết của tài khoản có số là 57222
+Xem chi tiết 45165</t>
+  </si>
+  <si>
+    <t>Liệt kê các giao dịch phát sinh từ ngày 2025-11-19 tới ngày hôm nay
+Những tài khoản nào diễn ra từ 2025-11-24 đến hôm nay?
+Xem biến động tài khoản giữa 2025-12-26 và hôm nay
+Lịch sử tài khoản 2025-02-08 đến hôm nay
+Sao kê tài khoản từ 2025-06-27 - hôm nay
+Truy xuất lịch sử tài khoản trong khoảng thời gian từ 2025-12-03 đến hôm nay
+Kiểm tra tài khoản trong ngày 2025-12-02</t>
+  </si>
+  <si>
+    <t>Vui lòng Tra cứu thông tin chi tiết của tài khoản có mã chi nhánh nơi quản lý tài khoản này. là 4920891957011
+Thông tin về tài khoản số 8372738178352
+Tra cứu tài khoản theo mã chi nhánh nơi quản lý tài khoản này. 4394484846255
+Hãy hiển thị dữ liệu bản ghi tài khoản với mã chi nhánh nơi quản lý tài khoản này. 3755342538790
+Xem chi tiết 4799880013753
+Tìm kiếm tài khoản ứng với số 4724630599038
+Check mã chi nhánh nơi quản lý tài khoản này. 1553414809905
+mã chi nhánh nơi quản lý tài khoản này. 7838732640846 là của ai?
+tài khoản 7172676252057</t>
+  </si>
+  <si>
+    <t>ví dụ: 411122****1234 4448405347748535 là của ai?
+Check ví dụ: 411122****1234 4841610459188582
+Tra cứu tài khoản theo ví dụ: 411122****1234 5746590403337035
+Hãy hiển thị dữ liệu bản ghi tài khoản với ví dụ: 411122****1234 5897198596610059
+Tìm kiếm tài khoản ứng với số 4662055474522759
+Thông tin về tài khoản số 5285512809070618
+Xem chi tiết 4883901492653984
+Vui lòng Tra cứu thông tin chi tiết của tài khoản có ví dụ: 411122****1234 là 5845368343965626
+tài khoản 5809020656554021</t>
+  </si>
+  <si>
+    <t>Hãy hiển thị dữ liệu bản ghi tài khoản với số 25017
+Tra cứu tài khoản theo số 50079
+Tìm kiếm tài khoản ứng với số 93489
+Xem chi tiết 48338
+Thông tin về tài khoản số 75402
+Check số 50036
+tài khoản 42707
+số 29615 là của ai?
+Vui lòng Tra cứu thông tin chi tiết của tài khoản có số là 91911</t>
+  </si>
+  <si>
+    <t>Tìm kiếm tài khoản ứng với số 45264
+Hãy hiển thị dữ liệu bản ghi tài khoản với số 20064
+số 20944 là của ai?
+Check số 65052
+Thông tin về tài khoản số 73783
+Xem chi tiết 50961
+tài khoản 59501
+Tra cứu tài khoản theo số 47389
+Vui lòng Tra cứu thông tin chi tiết của tài khoản có số là 81203</t>
+  </si>
+  <si>
+    <t>Xem biến động tài khoản giữa 2025-06-29 và hôm nay
+Lịch sử tài khoản 2025-02-02 đến hôm nay
+Liệt kê các giao dịch phát sinh từ ngày 2025-10-02 tới ngày hôm nay
+Những tài khoản nào diễn ra từ 2025-06-14 đến hôm nay?
+Truy xuất lịch sử tài khoản trong khoảng thời gian từ 2025-11-27 đến hôm nay
+Kiểm tra tài khoản trong ngày 2025-03-21
+Sao kê tài khoản từ 2025-06-16 - hôm nay</t>
+  </si>
+  <si>
+    <t>Lọc các tài khoản nào diễn ra từ 2025-04-05 đến hôm nay
+Liệt kê tài khoản đang phát sinh ngày 2026-01-20
+Sao kê tài khoản loại các từ ngày 2025-01-29 tới hôm nay
+Xem tài khoản có account_class là giữa trong khoảng 2025-08-17 - hôm nay
+Tìm tài khoản cho hôm 2025-10-16</t>
+  </si>
+  <si>
+    <t>id, khóa chính, tìm kiếm</t>
+  </si>
+  <si>
+    <t>core_customer_id, số, tìm kiếm</t>
+  </si>
+  <si>
+    <t>account_no, số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch., tìm kiếm</t>
+  </si>
+  <si>
+    <t>account_class, ví dụ: tài khoản thanh toán, tài khoản tiết kiệm, thẻ tín dụng..., danh sách</t>
+  </si>
+  <si>
+    <t>order_no, số thứ tự hiển thị tài khoản trên giao diện, tìm kiếm</t>
+  </si>
+  <si>
+    <t>status, trạng thái tài khoản, danh sách</t>
+  </si>
+  <si>
+    <t>verify_status, kết quả, danh sách</t>
+  </si>
+  <si>
+    <t>check_status, trạng thái kiểm tra, danh sách</t>
+  </si>
+  <si>
+    <t>channel_id, số, tìm kiếm</t>
+  </si>
+  <si>
+    <t>create_date, thời gian, ngày tháng</t>
+  </si>
+  <si>
+    <t>account_branch, mã chi nhánh nơi quản lý tài khoản này., tìm kiếm</t>
+  </si>
+  <si>
+    <t>card_mask, ví dụ: 411122****1234, tìm kiếm</t>
+  </si>
+  <si>
+    <t>customer_no, số, tìm kiếm</t>
+  </si>
+  <si>
+    <t>system_id, số, tìm kiếm</t>
+  </si>
+  <si>
+    <t>end_date, thời gian, ngày tháng</t>
+  </si>
+  <si>
+    <t>account_class, create_date, lọc đa điều kiện</t>
   </si>
   <si>
     <t>{"raw_text": "SELECT * FROM customer_account WHERE id = '{{id}}'"}</t>
@@ -430,6 +354,9 @@
   </si>
   <si>
     <t>{"raw_text": "SELECT * FROM customer_account WHERE end_date BETWEEN '{{start_date}}' AND '{{end_date}}' ORDER BY end_date DESC"}</t>
+  </si>
+  <si>
+    <t>{"raw_text": "SELECT * FROM customer_account WHERE account_class = '{{account_class}}' AND create_date BETWEEN '{{start_date}}' AND '{{end_date}}'"}</t>
   </si>
 </sst>
 </file>
@@ -787,7 +714,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -812,16 +739,16 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C2" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="D2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -829,16 +756,16 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -846,16 +773,16 @@
         <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="D4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -863,16 +790,16 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C5" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -880,16 +807,16 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C6" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="D6" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -897,16 +824,16 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C7" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="D7" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -914,16 +841,16 @@
         <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C8" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D8" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -931,134 +858,151 @@
         <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C9" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="D9" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="C10" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="D10" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="E10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C11" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="D11" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C12" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="D12" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C13" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D13" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="B14" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="C14" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="D14" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B15" t="s">
         <v>18</v>
       </c>
-      <c r="B15" t="s">
-        <v>33</v>
-      </c>
       <c r="C15" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D15" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E15" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C16" t="s">
         <v>43</v>
       </c>
       <c r="D16" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E16" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" t="s">
+        <v>60</v>
+      </c>
+      <c r="E17" t="s">
         <v>76</v>
       </c>
     </row>

</xml_diff>